<commit_message>
KPIs, Pie chart and bar chart
</commit_message>
<xml_diff>
--- a/DataSource/Qlik2PBI.xlsx
+++ b/DataSource/Qlik2PBI.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://keyrusgroup-my.sharepoint.com/personal/iuri_raposo_keyrus_com/Documents/Documents/Case Studies/Asset Management/DataSource/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D4EF1BD4-5991-4857-ACB1-7969C4FF6342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="8_{D4EF1BD4-5991-4857-ACB1-7969C4FF6342}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BF42262-A8DC-43FB-B412-0902B2CB81F3}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{B2CA230F-BA97-4E68-A392-CB3F5D1543A3}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Expression&amp;Measures" sheetId="1" r:id="rId1"/>
+    <sheet name="UI" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
   <si>
     <t>Qlik</t>
   </si>
@@ -54,6 +55,58 @@
   </si>
   <si>
     <t>Sum ({&lt;[Asset Class] = {'Equity'}&gt;} Asset_USD) / Sum ({&lt;[Asset Class] = &gt;} Asset_USD)</t>
+  </si>
+  <si>
+    <t>AUM_Total = 
+VAR SelectedCurrency = SELECTEDVALUE('Currency'[Currency Abr Name])
+RETURN 
+    SWITCH(SelectedCurrency,
+        "USD",  "$" &amp; ROUND(SUM(AUM[Asset_USD])/1000000000, 2),
+        "EUR", "€" &amp;ROUND(SUM(AUM[Asset_EUR])/1000000000,2),
+        "GBP", "£" &amp; ROUND(SUM(AUM[Asset_GBP])/1000000000,2),
+        ROUND(SUM(AUM[Asset_USD])/1000000000,2) --Default
+    ) &amp; "" &amp; "bn"</t>
+  </si>
+  <si>
+    <t>% Equity = 
+DIVIDE(
+    CALCULATE(
+        SUM(AUM[Asset_USD]),
+         AUM[Asset Class] = "Equity"
+    ),
+    CALCULATE(
+        SUM(AUM[Asset_USD]),
+        ALL(AUM[Asset Class]),
+        AUM[Asset Class]&lt;&gt;BLANK()
+    )
+)</t>
+  </si>
+  <si>
+    <t>UI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filter Panel </t>
+  </si>
+  <si>
+    <t>Container =&gt; Lisbox (Hide &amp; Show Contiditon)</t>
+  </si>
+  <si>
+    <t>Shape =&gt; Slicer =&gt; Bookmarks set up</t>
+  </si>
+  <si>
+    <t>% Equity</t>
+  </si>
+  <si>
+    <t>=Minstring({&lt; Asset_USD = {$(=Num(Max({&lt;[Asset Class] = {'Equity'}&gt;} Asset_USD)))} &gt;} [Account Name])</t>
+  </si>
+  <si>
+    <t>Highest Asset Invested</t>
+  </si>
+  <si>
+    <t>Highest Asset Invested = CALCULATE(
+                            Min(AUM[Account Name]),
+                            AUM[Asset_USD] = MAX(AUM[Asset_USD])
+)</t>
   </si>
 </sst>
 </file>
@@ -97,10 +150,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -435,12 +494,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C3EC172-CC21-471C-A474-2DF7463CA642}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="69.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.54296875" customWidth="1"/>
+    <col min="1" max="1" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="88.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="56.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
@@ -450,25 +509,82 @@
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" ht="145" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C2" s="4" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" ht="174" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
       <c r="B3" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="58" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{884CECC1-5636-48D0-A2C7-1EEFAEE43027}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="31.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>